<commit_message>
add feature authorization 1-1
</commit_message>
<xml_diff>
--- a/src/utils/athlete_import_example.xlsx
+++ b/src/utils/athlete_import_example.xlsx
@@ -433,7 +433,7 @@
         <v>phone</v>
       </c>
       <c r="E1" t="str">
-        <v>dob(mm/dd/yyyy)</v>
+        <v>dob(yyyy-mm-dd)</v>
       </c>
       <c r="F1" t="str">
         <v>gender</v>
@@ -486,7 +486,7 @@
         <v>0909123456</v>
       </c>
       <c r="E2" t="str">
-        <v>03/15/1990</v>
+        <v>1990-03-15</v>
       </c>
       <c r="F2" t="str">
         <v>M</v>
@@ -539,7 +539,7 @@
         <v>0987654321</v>
       </c>
       <c r="E3" t="str">
-        <v>12/01/1995</v>
+        <v>1995-12-01</v>
       </c>
       <c r="F3" t="str">
         <v>F</v>
@@ -618,13 +618,13 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>dob(mm/dd/yyyy) hoac dob</v>
+        <v>dob(yyyy-mm-dd) hoac dob</v>
       </c>
       <c r="B3" t="str">
         <v>Khong</v>
       </c>
       <c r="C3" t="str">
-        <v>Ngay sinh; co the dung cot dob thay cho dob(mm/dd/yyyy).</v>
+        <v>Ngay sinh: chuoi yyyy-mm-dd hoac o Date trong Excel; khong dung text dang dd/mm/yyyy.</v>
       </c>
     </row>
     <row r="4">

</xml_diff>